<commit_message>
Ajustes finales al README y evidencias para entrega.
</commit_message>
<xml_diff>
--- a/docs/Diccionario_Datos_Salud.xlsx
+++ b/docs/Diccionario_Datos_Salud.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edgar\Documents\PRUEBA TECNICA DATOS SERSOCIAL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edgar\Documents\PRUEBA TECNICA DATOS SERSOCIAL\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BAD12B9-2961-43A4-8040-8BA6EDED9BA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8E9F481-D41C-4C54-B9C1-BF220799340A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="178">
   <si>
     <t>Tabla/Vista</t>
   </si>
@@ -304,37 +304,256 @@
     <t>Campo temporal</t>
   </si>
   <si>
-    <t>core.vw_capacidad_por_prestador</t>
-  </si>
-  <si>
-    <t>capacidad_total</t>
-  </si>
-  <si>
-    <t>Total agregado de capacidad instalada por prestador y servicio</t>
-  </si>
-  <si>
-    <t>SUM fact_capacidad_instalada.capacidad_cantidad</t>
-  </si>
-  <si>
-    <t>Agregación GROUP BY</t>
-  </si>
-  <si>
-    <t>Métrica agregada</t>
-  </si>
-  <si>
-    <t>core.vw_capacidad_por_departamento</t>
-  </si>
-  <si>
-    <t>Total agregado de capacidad instalada por departamento</t>
-  </si>
-  <si>
-    <t>core.vw_capacidad_detalle</t>
-  </si>
-  <si>
-    <t>Detalle individual de capacidad instalada por servicio</t>
-  </si>
-  <si>
-    <t>fact_capacidad_instalada.capacidad_cantidad</t>
+    <t>core.vw_perfil_detallado_prestadores</t>
+  </si>
+  <si>
+    <t>Nombre_Institucion</t>
+  </si>
+  <si>
+    <t>NVARCHAR(255)</t>
+  </si>
+  <si>
+    <t>Razón social del prestador</t>
+  </si>
+  <si>
+    <t>Texto</t>
+  </si>
+  <si>
+    <t>Join por prestador_id</t>
+  </si>
+  <si>
+    <t>Numero_NIT</t>
+  </si>
+  <si>
+    <t>VARCHAR(20)</t>
+  </si>
+  <si>
+    <t>NIT oficial de la entidad</t>
+  </si>
+  <si>
+    <t>Formato numérico</t>
+  </si>
+  <si>
+    <t>Selección directa</t>
+  </si>
+  <si>
+    <t>Clase_IPS</t>
+  </si>
+  <si>
+    <t>NVARCHAR(100)</t>
+  </si>
+  <si>
+    <t>Categoría de prestador (REPS)</t>
+  </si>
+  <si>
+    <t>IPS, Profesional Ind., etc.</t>
+  </si>
+  <si>
+    <t>Naturaleza_Legal</t>
+  </si>
+  <si>
+    <t>Régimen jurídico de la entidad</t>
+  </si>
+  <si>
+    <t>Privada, Pública, Mixta</t>
+  </si>
+  <si>
+    <t>Descripcion_Servicio</t>
+  </si>
+  <si>
+    <t>NVARCHAR(500)</t>
+  </si>
+  <si>
+    <t>Nombre del servicio habilitado</t>
+  </si>
+  <si>
+    <t>Catálogo CIIPS</t>
+  </si>
+  <si>
+    <t>Cantidad_Reportada</t>
+  </si>
+  <si>
+    <t>Unidades de capacidad</t>
+  </si>
+  <si>
+    <t>Enteros &gt; 0</t>
+  </si>
+  <si>
+    <t>Fecha_Ultimo_Reporte</t>
+  </si>
+  <si>
+    <t>Vigencia del dato reportado</t>
+  </si>
+  <si>
+    <t>Fechas válidas</t>
+  </si>
+  <si>
+    <t>core.vw_estado_operativo_red_salud</t>
+  </si>
+  <si>
+    <t>Institucion</t>
+  </si>
+  <si>
+    <t>Nombre del prestador</t>
+  </si>
+  <si>
+    <t>Join</t>
+  </si>
+  <si>
+    <t>Tipo_Prestador</t>
+  </si>
+  <si>
+    <t>Clase de prestador</t>
+  </si>
+  <si>
+    <t>Catálogo REPS</t>
+  </si>
+  <si>
+    <t>Grupo_Servicio</t>
+  </si>
+  <si>
+    <t>Servicio analizado</t>
+  </si>
+  <si>
+    <t>Unidades</t>
+  </si>
+  <si>
+    <t>Capacidad física</t>
+  </si>
+  <si>
+    <t>Fecha_Corte</t>
+  </si>
+  <si>
+    <t>Fecha del reporte</t>
+  </si>
+  <si>
+    <t>Semaforo_Vigencia</t>
+  </si>
+  <si>
+    <t>NVARCHAR(50)</t>
+  </si>
+  <si>
+    <t>Clasificación de frescura del dato</t>
+  </si>
+  <si>
+    <t>Vigente, Requiere Act., Desactualizada</t>
+  </si>
+  <si>
+    <t>Calculado</t>
+  </si>
+  <si>
+    <t>DATEDIFF entre Fecha_Corte y GETDATE()</t>
+  </si>
+  <si>
+    <t>core.vw_resumen_capacidad_por_municipio</t>
+  </si>
+  <si>
+    <t>Departamento</t>
+  </si>
+  <si>
+    <t>NVARCHAR(150)</t>
+  </si>
+  <si>
+    <t>Join jerárquico</t>
+  </si>
+  <si>
+    <t>Municipio</t>
+  </si>
+  <si>
+    <t>Tipo_Servicio</t>
+  </si>
+  <si>
+    <t>Descripción del servicio</t>
+  </si>
+  <si>
+    <t>Total_Unidades_Disponibles</t>
+  </si>
+  <si>
+    <t>Sumatoria de capacidad</t>
+  </si>
+  <si>
+    <t>Enteros positivos</t>
+  </si>
+  <si>
+    <t>SUM(capacidad_cantidad)</t>
+  </si>
+  <si>
+    <t>Numero_IPS_Reportando</t>
+  </si>
+  <si>
+    <t>Conteo único de prestadores</t>
+  </si>
+  <si>
+    <t>COUNT(DISTINCT prestador_id)</t>
+  </si>
+  <si>
+    <t>staging.vw_resumen_rechazos_calidad</t>
+  </si>
+  <si>
+    <t>Origen_Dato</t>
+  </si>
+  <si>
+    <t>VARCHAR(100)</t>
+  </si>
+  <si>
+    <t>Tabla que generó el rechazo</t>
+  </si>
+  <si>
+    <t>stg_reps, stg_ciips</t>
+  </si>
+  <si>
+    <t>staging.stg_rechazos</t>
+  </si>
+  <si>
+    <t>Tipo_Error</t>
+  </si>
+  <si>
+    <t>Categoría del fallo de calidad</t>
+  </si>
+  <si>
+    <t>NIT_NULO, NO_REPS, etc.</t>
+  </si>
+  <si>
+    <t>ISNULL(motivo_rechazo, '...')</t>
+  </si>
+  <si>
+    <t>Total_Registros</t>
+  </si>
+  <si>
+    <t>Cantidad de filas afectadas</t>
+  </si>
+  <si>
+    <t>COUNT(*)</t>
+  </si>
+  <si>
+    <t>Ultima_Incidencia</t>
+  </si>
+  <si>
+    <t>DATETIME</t>
+  </si>
+  <si>
+    <t>Fecha del último error detectado</t>
+  </si>
+  <si>
+    <t>Fecha/Hora</t>
+  </si>
+  <si>
+    <t>MAX(fecha_rechazo)</t>
+  </si>
+  <si>
+    <t>Porcentaje_Impacto</t>
+  </si>
+  <si>
+    <t>DECIMAL(5,2)</t>
+  </si>
+  <si>
+    <t>Peso del error sobre el total</t>
+  </si>
+  <si>
+    <t>0.00 - 100.00</t>
+  </si>
+  <si>
+    <t>(COUNT / SUM OVER) * 100</t>
   </si>
 </sst>
 </file>
@@ -370,13 +589,53 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="12">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -387,6 +646,25 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C4FA83A7-6689-49AD-9534-223DF4453970}" name="Tabla1" displayName="Tabla1" ref="A1:J38" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <autoFilter ref="A1:J38" xr:uid="{C4FA83A7-6689-49AD-9534-223DF4453970}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{80F69618-6C06-47DB-93CE-DF981C3CAC40}" name="Tabla/Vista" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{2B700612-2735-4049-85F0-6136B5230B39}" name="Nombre del campo" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{317A0F49-AE92-44DB-8D10-57FDC3B5C4F1}" name="Tipo de dato" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{0A3787CB-2483-43FE-905D-606C6C3149D1}" name="Descripción funcional" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{579B3361-868C-4245-99F8-CB73A382C459}" name="Valores permitidos" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{E6003DD6-3D6C-45DB-8BEB-3949099AC582}" name="¿Puede ser nulo?" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{A0F35725-B13A-495F-8BF8-FD6ECBECE0FA}" name="Origen" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{5BA8C1B1-950A-4516-8CC6-412E32ADE71B}" name="Transformación aplicada" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{66BDA29C-D1FA-4FF8-92C2-61304B6484EB}" name="¿Es campo clave?" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{EDF31D44-2AD0-4EF8-8FE7-2D49B8CF10FF}" name="¿Es dato sensible?" dataDxfId="2"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -674,597 +952,1243 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="56.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="40.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="60.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="45.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="56.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="40.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.42578125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="60.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="45.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.28515625" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="F2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="F3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="I3" t="s">
-        <v>15</v>
-      </c>
-      <c r="J3" t="s">
+      <c r="I3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="F4" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="F4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="F5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="I5" t="s">
-        <v>15</v>
-      </c>
-      <c r="J5" t="s">
+      <c r="I5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J5" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="A6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F6" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="F6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="J6" t="s">
+      <c r="J6" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="A7" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="F7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" t="s">
+      <c r="F7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J7" t="s">
+      <c r="J7" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="A8" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" t="s">
+      <c r="F8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="H8" t="s">
+      <c r="H8" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="I8" t="s">
+      <c r="I8" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="J8" t="s">
+      <c r="J8" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="A9" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" t="s">
+      <c r="F9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I9" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="J9" t="s">
+      <c r="J9" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="A10" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="I10" t="s">
-        <v>15</v>
-      </c>
-      <c r="J10" t="s">
+      <c r="I10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J10" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="A11" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="F11" t="s">
-        <v>15</v>
-      </c>
-      <c r="G11" t="s">
+      <c r="F11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G11" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="I11" t="s">
+      <c r="I11" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="J11" t="s">
+      <c r="J11" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="A12" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="F12" t="s">
-        <v>15</v>
-      </c>
-      <c r="G12" t="s">
+      <c r="F12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G12" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="H12" t="s">
+      <c r="H12" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="I12" t="s">
+      <c r="I12" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="J12" t="s">
+      <c r="J12" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="A13" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="F13" t="s">
-        <v>15</v>
-      </c>
-      <c r="G13" t="s">
+      <c r="F13" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G13" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="H13" t="s">
+      <c r="H13" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="I13" t="s">
-        <v>15</v>
-      </c>
-      <c r="J13" t="s">
+      <c r="I13" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J13" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="A14" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="F14" t="s">
-        <v>15</v>
-      </c>
-      <c r="G14" t="s">
+      <c r="F14" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G14" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H14" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="I14" t="s">
+      <c r="I14" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="J14" t="s">
+      <c r="J14" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="A15" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H15" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="I15" t="s">
+      <c r="I15" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="J15" t="s">
+      <c r="J15" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="A16" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D21" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="E16" t="s">
-        <v>82</v>
-      </c>
-      <c r="F16" t="s">
-        <v>15</v>
-      </c>
-      <c r="G16" t="s">
-        <v>97</v>
-      </c>
-      <c r="H16" t="s">
+      <c r="D23" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="I16" t="s">
-        <v>99</v>
-      </c>
-      <c r="J16" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>100</v>
-      </c>
-      <c r="B17" t="s">
-        <v>95</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="F23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C26" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D17" t="s">
-        <v>101</v>
-      </c>
-      <c r="E17" t="s">
-        <v>82</v>
-      </c>
-      <c r="F17" t="s">
-        <v>15</v>
-      </c>
-      <c r="G17" t="s">
-        <v>97</v>
-      </c>
-      <c r="H17" t="s">
+      <c r="D26" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="I17" t="s">
-        <v>99</v>
-      </c>
-      <c r="J17" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>102</v>
-      </c>
-      <c r="B18" t="s">
-        <v>80</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="F29" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C32" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D18" t="s">
-        <v>103</v>
-      </c>
-      <c r="E18" t="s">
-        <v>82</v>
-      </c>
-      <c r="F18" t="s">
-        <v>15</v>
-      </c>
-      <c r="G18" t="s">
+      <c r="D32" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="H34" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="H18" t="s">
-        <v>79</v>
-      </c>
-      <c r="I18" t="s">
-        <v>15</v>
-      </c>
-      <c r="J18" t="s">
+      <c r="I34" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J34" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J36" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J38" s="1" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>